<commit_message>
Release v2.1.0 aggregate evidence and corrected pilot
</commit_message>
<xml_diff>
--- a/Context_Engineering_Evidence_Explorer.xlsx
+++ b/Context_Engineering_Evidence_Explorer.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Re127c775a5f44225"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pooled" sheetId="2" r:id="R5313f5cf60b9489c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station Effects" sheetId="3" r:id="Rb7be1c64a0cb40a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equal Station" sheetId="4" r:id="R23d51da9fa0f4211"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Archive Batch" sheetId="5" r:id="Re28377e4ca774c02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Bins" sheetId="6" r:id="R00fbb32abeb84727"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inheritance" sheetId="7" r:id="R1d9cfd3259084559"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Frame" sheetId="8" r:id="R6e0d7be9e6e24856"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aggregate Catalog" sheetId="9" r:id="Ra5a270ca6c054600"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Claims" sheetId="10" r:id="R16b4fee264264f37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Lineage" sheetId="11" r:id="R22f7c2ec4dba46d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Receipts" sheetId="12" r:id="R37bb80ba165e4275"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="13" r:id="R22ba211fb77746af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Summary" sheetId="14" r:id="R80b370569ed24006"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Headline Checks" sheetId="15" r:id="R48203f3063a34419"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rf26796d29bd844e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pooled" sheetId="2" r:id="Rc2fec34f8228426c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station Effects" sheetId="3" r:id="R1fe796cd1ef74d72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equal Station" sheetId="4" r:id="Raab7952bb06f4078"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Archive Batch" sheetId="5" r:id="R2af84eeadb534506"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Bins" sheetId="6" r:id="Reb8ffadbc32c4275"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inheritance" sheetId="7" r:id="R087699440d7347ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Frame" sheetId="8" r:id="R55d86a61ea3e4eb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aggregate Catalog" sheetId="9" r:id="R4a37c58029254e36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Claims" sheetId="10" r:id="Reffff0fb96384dd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Lineage" sheetId="11" r:id="R4e16ea52e40e4185"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Receipts" sheetId="12" r:id="R2edafd8df1614f15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="13" r:id="Ra3a6cc4e9071461f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action Summary" sheetId="14" r:id="R65b9fe6cb2524186"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Headline Checks" sheetId="15" r:id="Rf2be004dd40441cf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -654,7 +654,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="124" name="SourceFrameTable" displayName="SourceFrameTable" ref="A1:G146" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="124" name="SourceFrameTable" displayName="SourceFrameTable" ref="A1:G183" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="item_id"/>
     <x:tableColumn id="2" name="scope"/>
@@ -1394,7 +1394,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7150dbc18c0b4e45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9585893090c84212"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2200,7 +2200,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84b25a6ee2b34105"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8dbb1ebf7624578"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2490,7 +2490,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e92879b9cee48ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67393b9f5a24463d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5616,7 +5616,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ca5134dca364ffd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fa8c919b9fc4309"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5729,7 +5729,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b11fcd21fd54951"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29b78b9c9efb4f1f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6637,7 +6637,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb36e7932e83742e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd5fbd16029c4cca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14474,7 +14474,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ef815d41c9b4b54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e7aec403da042f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15222,7 +15222,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc4bfea4386b4853"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb52950a65a3c488e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16654,7 +16654,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60a9fefc360846d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd66446d5298444f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17099,7 +17099,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0671ed97b17543d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96f442f047034397"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17137,16 +17137,16 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B2" s="38" t="n">
-        <x:v>1860</x:v>
+        <x:v>1859</x:v>
       </x:c>
       <x:c r="C2" s="38" t="n">
         <x:v>2560</x:v>
       </x:c>
       <x:c r="D2" s="37" t="n">
-        <x:v>0.7265625</x:v>
+        <x:v>0.726171875</x:v>
       </x:c>
       <x:c r="E2" s="38" t="n">
-        <x:v>700</x:v>
+        <x:v>701</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -17154,16 +17154,16 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="38" t="n">
-        <x:v>2104</x:v>
+        <x:v>2103</x:v>
       </x:c>
       <x:c r="C3" s="38" t="n">
         <x:v>2560</x:v>
       </x:c>
       <x:c r="D3" s="37" t="n">
-        <x:v>0.821875</x:v>
+        <x:v>0.821484375</x:v>
       </x:c>
       <x:c r="E3" s="38" t="n">
-        <x:v>456</x:v>
+        <x:v>457</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -17220,7 +17220,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc9df04db6474375"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d496d7993694884"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17663,7 +17663,7 @@
         <x:v>high_confidence_candidates</x:v>
       </x:c>
       <x:c r="D19" s="38" t="n">
-        <x:v>1107</x:v>
+        <x:v>1106</x:v>
       </x:c>
       <x:c r="E19" s="13" t="str">
         <x:v>count</x:v>
@@ -17686,7 +17686,7 @@
         <x:v>probable_candidates</x:v>
       </x:c>
       <x:c r="D20" s="71" t="n">
-        <x:v>1149</x:v>
+        <x:v>1150</x:v>
       </x:c>
       <x:c r="E20" s="7" t="str">
         <x:v>count</x:v>
@@ -18043,7 +18043,7 @@
         <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="36" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A36" s="7" t="str">
         <x:v>FRAME-35</x:v>
       </x:c>
@@ -18054,7 +18054,7 @@
         <x:v>review46.changed_measurements_or_trajectory_count</x:v>
       </x:c>
       <x:c r="D36" s="71" t="n">
-        <x:v>18</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E36" s="7" t="str">
         <x:v>count</x:v>
@@ -18063,7 +18063,7 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G36" s="7" t="str">
-        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications</x:v>
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; source-measurement, derived-field or alias-membership changes; provenance-status-only transitions excluded</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -18089,7 +18089,7 @@
         <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="38" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A38" s="7" t="str">
         <x:v>FRAME-37</x:v>
       </x:c>
@@ -18097,10 +18097,10 @@
         <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C38" s="7" t="str">
-        <x:v>review46.distinct_v5_events</x:v>
+        <x:v>review46.current_primary_provenance_status_only_count</x:v>
       </x:c>
       <x:c r="D38" s="71" t="n">
-        <x:v>46</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E38" s="7" t="str">
         <x:v>count</x:v>
@@ -18109,10 +18109,10 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G38" s="7" t="str">
-        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; only provenance-status text changes; observed transition v2_codex_unchanged to resolved, with unchanged identity, aliases and tracked evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A39" s="7" t="str">
         <x:v>FRAME-38</x:v>
       </x:c>
@@ -18120,10 +18120,10 @@
         <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C39" s="7" t="str">
-        <x:v>review46.held_count</x:v>
+        <x:v>review46.current_primary_strict_status_inclusive_changed_count</x:v>
       </x:c>
       <x:c r="D39" s="71" t="n">
-        <x:v>0</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E39" s="7" t="str">
         <x:v>count</x:v>
@@ -18132,10 +18132,10 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G39" s="7" t="str">
-        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; strict equality includes exact provenance-status text, not just substantive evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A40" s="7" t="str">
         <x:v>FRAME-39</x:v>
       </x:c>
@@ -18143,10 +18143,10 @@
         <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C40" s="7" t="str">
-        <x:v>review46.historical_events</x:v>
+        <x:v>review46.current_primary_strict_status_inclusive_unchanged_count</x:v>
       </x:c>
       <x:c r="D40" s="71" t="n">
-        <x:v>46</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E40" s="7" t="str">
         <x:v>count</x:v>
@@ -18155,7 +18155,7 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G40" s="7" t="str">
-        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications</x:v>
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; strict equality includes exact provenance-status text, not just substantive evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -18166,10 +18166,10 @@
         <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C41" s="7" t="str">
-        <x:v>review46.same_measured_trajectory_and_labels_count</x:v>
+        <x:v>review46.distinct_v5_events</x:v>
       </x:c>
       <x:c r="D41" s="71" t="n">
-        <x:v>28</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="E41" s="7" t="str">
         <x:v>count</x:v>
@@ -18189,10 +18189,10 @@
         <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C42" s="7" t="str">
-        <x:v>review46.v5_primary_member_count</x:v>
+        <x:v>review46.held_count</x:v>
       </x:c>
       <x:c r="D42" s="71" t="n">
-        <x:v>39</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E42" s="7" t="str">
         <x:v>count</x:v>
@@ -18209,13 +18209,13 @@
         <x:v>FRAME-42</x:v>
       </x:c>
       <x:c r="B43" s="7" t="str">
-        <x:v>historical to current primary overlap</x:v>
+        <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C43" s="7" t="str">
-        <x:v>full_primary_overlap.absorbed_boundary_event_count</x:v>
+        <x:v>review46.historical_events</x:v>
       </x:c>
       <x:c r="D43" s="71" t="n">
-        <x:v>13</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="E43" s="7" t="str">
         <x:v>count</x:v>
@@ -18224,21 +18224,21 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G43" s="7" t="str">
-        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A44" s="7" t="str">
         <x:v>FRAME-43</x:v>
       </x:c>
       <x:c r="B44" s="7" t="str">
-        <x:v>historical to current primary overlap</x:v>
+        <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C44" s="7" t="str">
-        <x:v>full_primary_overlap.alias_membership_expanded_event_count</x:v>
+        <x:v>review46.provenance_status_only_count</x:v>
       </x:c>
       <x:c r="D44" s="71" t="n">
-        <x:v>51</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E44" s="7" t="str">
         <x:v>count</x:v>
@@ -18247,21 +18247,21 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G44" s="7" t="str">
-        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; only provenance-status text changes; observed transition v2_codex_unchanged to resolved, with unchanged identity, aliases and tracked evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A45" s="7" t="str">
         <x:v>FRAME-44</x:v>
       </x:c>
       <x:c r="B45" s="7" t="str">
-        <x:v>historical to current primary overlap</x:v>
+        <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C45" s="7" t="str">
-        <x:v>full_primary_overlap.changed_derived_labels_count</x:v>
+        <x:v>review46.same_measured_trajectory_and_labels_count</x:v>
       </x:c>
       <x:c r="D45" s="71" t="n">
-        <x:v>208</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="E45" s="7" t="str">
         <x:v>count</x:v>
@@ -18270,21 +18270,21 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G45" s="7" t="str">
-        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; substantive equality excludes provenance-status text and compares all 15 source fields, eight derived fields and alias membership</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A46" s="7" t="str">
         <x:v>FRAME-45</x:v>
       </x:c>
       <x:c r="B46" s="7" t="str">
-        <x:v>historical to current primary overlap</x:v>
+        <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C46" s="7" t="str">
-        <x:v>full_primary_overlap.changed_measurements_or_trajectory_count</x:v>
+        <x:v>review46.strict_status_inclusive_changed_count</x:v>
       </x:c>
       <x:c r="D46" s="71" t="n">
-        <x:v>467</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E46" s="7" t="str">
         <x:v>count</x:v>
@@ -18293,21 +18293,21 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G46" s="7" t="str">
-        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; strict equality includes exact provenance-status text, not just substantive evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A47" s="7" t="str">
         <x:v>FRAME-46</x:v>
       </x:c>
       <x:c r="B47" s="7" t="str">
-        <x:v>historical to current primary overlap</x:v>
+        <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C47" s="7" t="str">
-        <x:v>full_primary_overlap.condition_changed_among_current_primary_count</x:v>
+        <x:v>review46.strict_status_inclusive_unchanged_count</x:v>
       </x:c>
       <x:c r="D47" s="71" t="n">
-        <x:v>4</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E47" s="7" t="str">
         <x:v>count</x:v>
@@ -18316,7 +18316,7 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G47" s="7" t="str">
-        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; strict equality includes exact provenance-status text, not just substantive evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -18324,13 +18324,13 @@
         <x:v>FRAME-47</x:v>
       </x:c>
       <x:c r="B48" s="7" t="str">
-        <x:v>historical to current primary overlap</x:v>
+        <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C48" s="7" t="str">
-        <x:v>full_primary_overlap.direct_unchanged_id_primary_overlap</x:v>
+        <x:v>review46.v5_primary_member_count</x:v>
       </x:c>
       <x:c r="D48" s="71" t="n">
-        <x:v>758</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="E48" s="7" t="str">
         <x:v>count</x:v>
@@ -18339,21 +18339,21 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G48" s="7" t="str">
-        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A49" s="7" t="str">
         <x:v>FRAME-48</x:v>
       </x:c>
       <x:c r="B49" s="7" t="str">
-        <x:v>historical to current primary overlap</x:v>
+        <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C49" s="7" t="str">
-        <x:v>full_primary_overlap.distinct_v5_events</x:v>
+        <x:v>review46.disposition_counts.current_primary_changed</x:v>
       </x:c>
       <x:c r="D49" s="71" t="n">
-        <x:v>943</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E49" s="7" t="str">
         <x:v>count</x:v>
@@ -18362,21 +18362,21 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G49" s="7" t="str">
-        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; unchanged/changed uses substantive tracked-evidence equality, excluding status-only transitions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A50" s="7" t="str">
         <x:v>FRAME-49</x:v>
       </x:c>
       <x:c r="B50" s="7" t="str">
-        <x:v>historical to current primary overlap</x:v>
+        <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C50" s="7" t="str">
-        <x:v>full_primary_overlap.held_count</x:v>
+        <x:v>review46.disposition_counts.current_primary_unchanged</x:v>
       </x:c>
       <x:c r="D50" s="71" t="n">
-        <x:v>1</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E50" s="7" t="str">
         <x:v>count</x:v>
@@ -18385,7 +18385,7 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G50" s="7" t="str">
-        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; unchanged/changed uses substantive tracked-evidence equality, excluding status-only transitions</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -18393,13 +18393,13 @@
         <x:v>FRAME-50</x:v>
       </x:c>
       <x:c r="B51" s="7" t="str">
-        <x:v>historical to current primary overlap</x:v>
+        <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C51" s="7" t="str">
-        <x:v>full_primary_overlap.historical_events</x:v>
+        <x:v>review46.disposition_counts.not_current_primary</x:v>
       </x:c>
       <x:c r="D51" s="71" t="n">
-        <x:v>946</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E51" s="7" t="str">
         <x:v>count</x:v>
@@ -18408,21 +18408,21 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G51" s="7" t="str">
-        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A52" s="7" t="str">
         <x:v>FRAME-51</x:v>
       </x:c>
       <x:c r="B52" s="7" t="str">
-        <x:v>historical to current primary overlap</x:v>
+        <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C52" s="7" t="str">
-        <x:v>full_primary_overlap.same_measured_trajectory_and_labels_count</x:v>
+        <x:v>review46.change_category_counts.derived_label_change</x:v>
       </x:c>
       <x:c r="D52" s="71" t="n">
-        <x:v>479</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E52" s="7" t="str">
         <x:v>count</x:v>
@@ -18431,21 +18431,21 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G52" s="7" t="str">
-        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; mutually exclusive priority: derived labels, source measurements, aliases, status-only, strictly unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A53" s="7" t="str">
         <x:v>FRAME-52</x:v>
       </x:c>
       <x:c r="B53" s="7" t="str">
-        <x:v>historical to current primary overlap</x:v>
+        <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C53" s="7" t="str">
-        <x:v>full_primary_overlap.v3_primary_total</x:v>
+        <x:v>review46.change_category_counts.measurement_change_without_derived_label_change</x:v>
       </x:c>
       <x:c r="D53" s="71" t="n">
-        <x:v>946</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E53" s="7" t="str">
         <x:v>count</x:v>
@@ -18454,21 +18454,21 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G53" s="7" t="str">
-        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; mutually exclusive priority: derived labels, source measurements, aliases, status-only, strictly unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A54" s="7" t="str">
         <x:v>FRAME-53</x:v>
       </x:c>
       <x:c r="B54" s="7" t="str">
-        <x:v>historical to current primary overlap</x:v>
+        <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C54" s="7" t="str">
-        <x:v>full_primary_overlap.v5_primary_distinct_events_reached_from_v3_primary</x:v>
+        <x:v>review46.change_category_counts.provenance_status_only</x:v>
       </x:c>
       <x:c r="D54" s="71" t="n">
-        <x:v>774</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E54" s="7" t="str">
         <x:v>count</x:v>
@@ -18477,21 +18477,21 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G54" s="7" t="str">
-        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; only provenance-status text changes; observed transition v2_codex_unchanged to resolved, with unchanged identity, aliases and tracked evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A55" s="7" t="str">
         <x:v>FRAME-54</x:v>
       </x:c>
       <x:c r="B55" s="7" t="str">
-        <x:v>historical to current primary overlap</x:v>
+        <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C55" s="7" t="str">
-        <x:v>full_primary_overlap.v5_primary_events_not_reached_from_v3_primary</x:v>
+        <x:v>review46.change_category_counts.strictly_unchanged</x:v>
       </x:c>
       <x:c r="D55" s="71" t="n">
-        <x:v>84</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E55" s="7" t="str">
         <x:v>count</x:v>
@@ -18500,21 +18500,21 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G55" s="7" t="str">
-        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; strict equality includes exact provenance-status text, not just substantive evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A56" s="7" t="str">
         <x:v>FRAME-55</x:v>
       </x:c>
       <x:c r="B56" s="7" t="str">
-        <x:v>historical to current primary overlap</x:v>
+        <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C56" s="7" t="str">
-        <x:v>full_primary_overlap.v5_primary_member_count</x:v>
+        <x:v>review46.current_primary_change_category_counts.derived_label_change</x:v>
       </x:c>
       <x:c r="D56" s="71" t="n">
-        <x:v>776</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E56" s="7" t="str">
         <x:v>count</x:v>
@@ -18523,21 +18523,21 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G56" s="7" t="str">
-        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="57" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; mutually exclusive priority: derived labels, source measurements, aliases, status-only, strictly unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A57" s="7" t="str">
         <x:v>FRAME-56</x:v>
       </x:c>
       <x:c r="B57" s="7" t="str">
-        <x:v>historical to current primary overlap</x:v>
+        <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C57" s="7" t="str">
-        <x:v>full_primary_overlap.v5_primary_total</x:v>
+        <x:v>review46.current_primary_change_category_counts.measurement_change_without_derived_label_change</x:v>
       </x:c>
       <x:c r="D57" s="71" t="n">
-        <x:v>858</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E57" s="7" t="str">
         <x:v>count</x:v>
@@ -18546,21 +18546,21 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G57" s="7" t="str">
-        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="58" ht="15" hidden="0" customHeight="1">
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; mutually exclusive priority: derived labels, source measurements, aliases, status-only, strictly unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A58" s="7" t="str">
         <x:v>FRAME-57</x:v>
       </x:c>
       <x:c r="B58" s="7" t="str">
-        <x:v>historical operational evidence rejoin</x:v>
+        <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C58" s="7" t="str">
-        <x:v>historical_evidence_all138.distinct_v5_events</x:v>
+        <x:v>review46.current_primary_change_category_counts.provenance_status_only</x:v>
       </x:c>
       <x:c r="D58" s="71" t="n">
-        <x:v>138</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E58" s="7" t="str">
         <x:v>count</x:v>
@@ -18569,21 +18569,21 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G58" s="7" t="str">
-        <x:v>Operational evidence, not a representative classifier reference study</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="59" ht="15" hidden="0" customHeight="1">
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; only provenance-status text changes; observed transition v2_codex_unchanged to resolved, with unchanged identity, aliases and tracked evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A59" s="7" t="str">
         <x:v>FRAME-58</x:v>
       </x:c>
       <x:c r="B59" s="7" t="str">
-        <x:v>historical operational evidence rejoin</x:v>
+        <x:v>historical event-v3 author-check rejoin</x:v>
       </x:c>
       <x:c r="C59" s="7" t="str">
-        <x:v>historical_evidence_all138.distinct_v5_primary_events</x:v>
+        <x:v>review46.current_primary_change_category_counts.strictly_unchanged</x:v>
       </x:c>
       <x:c r="D59" s="71" t="n">
-        <x:v>5</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E59" s="7" t="str">
         <x:v>count</x:v>
@@ -18592,21 +18592,21 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G59" s="7" t="str">
-        <x:v>Operational evidence, not a representative classifier reference study</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="60" ht="15" hidden="0" customHeight="1">
+        <x:v>Historical case-level counts; no inferred transfer of confirmation to changed event-v5 classifications; strict equality includes exact provenance-status text, not just substantive evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A60" s="7" t="str">
         <x:v>FRAME-59</x:v>
       </x:c>
       <x:c r="B60" s="7" t="str">
-        <x:v>historical operational evidence rejoin</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C60" s="7" t="str">
-        <x:v>historical_evidence_all138.historical_records</x:v>
+        <x:v>full_primary_overlap.absorbed_boundary_event_count</x:v>
       </x:c>
       <x:c r="D60" s="71" t="n">
-        <x:v>138</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E60" s="7" t="str">
         <x:v>count</x:v>
@@ -18615,7 +18615,7 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G60" s="7" t="str">
-        <x:v>Operational evidence, not a representative classifier reference study</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -18623,13 +18623,13 @@
         <x:v>FRAME-60</x:v>
       </x:c>
       <x:c r="B61" s="7" t="str">
-        <x:v>historical operational evidence rejoin</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C61" s="7" t="str">
-        <x:v>historical_evidence_all138.historical_records_mapping_to_v5_primary</x:v>
+        <x:v>full_primary_overlap.alias_membership_expanded_event_count</x:v>
       </x:c>
       <x:c r="D61" s="71" t="n">
-        <x:v>5</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="E61" s="7" t="str">
         <x:v>count</x:v>
@@ -18638,7 +18638,7 @@
         <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G61" s="7" t="str">
-        <x:v>Operational evidence, not a representative classifier reference study</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -18646,45 +18646,45 @@
         <x:v>FRAME-61</x:v>
       </x:c>
       <x:c r="B62" s="7" t="str">
-        <x:v>event-v4 to event-v5 native identity accounting</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C62" s="7" t="str">
-        <x:v>invariants.native_invariant_checks</x:v>
+        <x:v>full_primary_overlap.changed_derived_labels_count</x:v>
       </x:c>
       <x:c r="D62" s="71" t="n">
-        <x:v>3948491</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="E62" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F62" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G62" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="63" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A63" s="7" t="str">
         <x:v>FRAME-62</x:v>
       </x:c>
       <x:c r="B63" s="7" t="str">
-        <x:v>event-v4 to event-v5 native identity accounting</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C63" s="7" t="str">
-        <x:v>invariants.unchanged_native_event_identities</x:v>
+        <x:v>full_primary_overlap.changed_measurements_or_trajectory_count</x:v>
       </x:c>
       <x:c r="D63" s="71" t="n">
-        <x:v>20965</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="E63" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F63" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G63" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; source-measurement, derived-field or alias-membership changes; provenance-status-only transitions excluded</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -18692,91 +18692,91 @@
         <x:v>FRAME-63</x:v>
       </x:c>
       <x:c r="B64" s="7" t="str">
-        <x:v>event-v4 to event-v5 automated disposition</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C64" s="7" t="str">
-        <x:v>status_transitions.quarantined-&gt;quarantined</x:v>
+        <x:v>full_primary_overlap.condition_changed_among_current_primary_count</x:v>
       </x:c>
       <x:c r="D64" s="71" t="n">
-        <x:v>283</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E64" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F64" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G64" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="65" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A65" s="7" t="str">
         <x:v>FRAME-64</x:v>
       </x:c>
       <x:c r="B65" s="7" t="str">
-        <x:v>event-v4 to event-v5 automated disposition</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C65" s="7" t="str">
-        <x:v>status_transitions.resolved-&gt;resolved</x:v>
+        <x:v>full_primary_overlap.current_primary_provenance_status_only_count</x:v>
       </x:c>
       <x:c r="D65" s="71" t="n">
-        <x:v>20682</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="E65" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F65" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G65" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="66" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; only provenance-status text changes; observed transition v2_codex_unchanged to resolved, with unchanged identity, aliases and tracked evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A66" s="7" t="str">
         <x:v>FRAME-65</x:v>
       </x:c>
       <x:c r="B66" s="7" t="str">
-        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C66" s="7" t="str">
-        <x:v>measurement_changes.automated_disposition_changed_events</x:v>
+        <x:v>full_primary_overlap.current_primary_strict_status_inclusive_changed_count</x:v>
       </x:c>
       <x:c r="D66" s="71" t="n">
-        <x:v>339</x:v>
+        <x:v>344</x:v>
       </x:c>
       <x:c r="E66" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F66" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G66" s="7" t="str">
-        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="67" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; strict equality includes exact provenance-status text, not just substantive evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A67" s="7" t="str">
         <x:v>FRAME-66</x:v>
       </x:c>
       <x:c r="B67" s="7" t="str">
-        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C67" s="7" t="str">
-        <x:v>measurement_changes.completed_substantive_action_calls_changed_events</x:v>
+        <x:v>full_primary_overlap.current_primary_strict_status_inclusive_unchanged_count</x:v>
       </x:c>
       <x:c r="D67" s="71" t="n">
-        <x:v>1522</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="E67" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F67" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G67" s="7" t="str">
-        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; strict equality includes exact provenance-status text, not just substantive evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -18784,22 +18784,22 @@
         <x:v>FRAME-67</x:v>
       </x:c>
       <x:c r="B68" s="7" t="str">
-        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C68" s="7" t="str">
-        <x:v>measurement_changes.context_mode_mask_changed_events</x:v>
+        <x:v>full_primary_overlap.direct_unchanged_id_primary_overlap</x:v>
       </x:c>
       <x:c r="D68" s="71" t="n">
-        <x:v>21</x:v>
+        <x:v>758</x:v>
       </x:c>
       <x:c r="E68" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F68" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G68" s="7" t="str">
-        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -18807,22 +18807,22 @@
         <x:v>FRAME-68</x:v>
       </x:c>
       <x:c r="B69" s="7" t="str">
-        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C69" s="7" t="str">
-        <x:v>measurement_changes.context_trace_status_changed_events</x:v>
+        <x:v>full_primary_overlap.distinct_v5_events</x:v>
       </x:c>
       <x:c r="D69" s="71" t="n">
-        <x:v>377</x:v>
+        <x:v>943</x:v>
       </x:c>
       <x:c r="E69" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F69" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G69" s="7" t="str">
-        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -18830,22 +18830,22 @@
         <x:v>FRAME-69</x:v>
       </x:c>
       <x:c r="B70" s="7" t="str">
-        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C70" s="7" t="str">
-        <x:v>measurement_changes.frontloading_changed_events</x:v>
+        <x:v>full_primary_overlap.held_count</x:v>
       </x:c>
       <x:c r="D70" s="71" t="n">
-        <x:v>13</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E70" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F70" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G70" s="7" t="str">
-        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -18853,114 +18853,114 @@
         <x:v>FRAME-70</x:v>
       </x:c>
       <x:c r="B71" s="7" t="str">
-        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C71" s="7" t="str">
-        <x:v>measurement_changes.prompt_artifact_reference_count_changed_events</x:v>
+        <x:v>full_primary_overlap.historical_events</x:v>
       </x:c>
       <x:c r="D71" s="71" t="n">
-        <x:v>130</x:v>
+        <x:v>946</x:v>
       </x:c>
       <x:c r="E71" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F71" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G71" s="7" t="str">
-        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="72" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A72" s="7" t="str">
         <x:v>FRAME-71</x:v>
       </x:c>
       <x:c r="B72" s="7" t="str">
-        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C72" s="7" t="str">
-        <x:v>measurement_changes.reclassified_calls</x:v>
+        <x:v>full_primary_overlap.provenance_status_only_count</x:v>
       </x:c>
       <x:c r="D72" s="71" t="n">
-        <x:v>6788</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="E72" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F72" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G72" s="7" t="str">
-        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="73" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; only provenance-status text changes; observed transition v2_codex_unchanged to resolved, with unchanged identity, aliases and tracked evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A73" s="7" t="str">
         <x:v>FRAME-72</x:v>
       </x:c>
       <x:c r="B73" s="7" t="str">
-        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C73" s="7" t="str">
-        <x:v>measurement_changes.successful_reclassified_calls</x:v>
+        <x:v>full_primary_overlap.same_measured_trajectory_and_labels_count</x:v>
       </x:c>
       <x:c r="D73" s="71" t="n">
-        <x:v>6780</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="E73" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F73" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G73" s="7" t="str">
-        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="74" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; substantive equality excludes provenance-status text and compares all 15 source fields, eight derived fields and alias membership</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A74" s="7" t="str">
         <x:v>FRAME-73</x:v>
       </x:c>
       <x:c r="B74" s="7" t="str">
-        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C74" s="7" t="str">
-        <x:v>measurement_changes.successful_todowrite_events</x:v>
+        <x:v>full_primary_overlap.strict_status_inclusive_changed_count</x:v>
       </x:c>
       <x:c r="D74" s="71" t="n">
-        <x:v>1522</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="E74" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F74" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G74" s="7" t="str">
-        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="75" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; strict equality includes exact provenance-status text, not just substantive evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A75" s="7" t="str">
         <x:v>FRAME-74</x:v>
       </x:c>
       <x:c r="B75" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C75" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.frontloading_changed.v4_primary_ce</x:v>
+        <x:v>full_primary_overlap.strict_status_inclusive_unchanged_count</x:v>
       </x:c>
       <x:c r="D75" s="71" t="n">
-        <x:v>2</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="E75" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F75" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G75" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; strict equality includes exact provenance-status text, not just substantive evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -18968,22 +18968,22 @@
         <x:v>FRAME-75</x:v>
       </x:c>
       <x:c r="B76" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C76" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.frontloading_changed.v4_resolved</x:v>
+        <x:v>full_primary_overlap.v3_primary_total</x:v>
       </x:c>
       <x:c r="D76" s="71" t="n">
-        <x:v>13</x:v>
+        <x:v>946</x:v>
       </x:c>
       <x:c r="E76" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F76" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G76" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -18991,22 +18991,22 @@
         <x:v>FRAME-76</x:v>
       </x:c>
       <x:c r="B77" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C77" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.frontloading_changed.v4_unrestricted_ce</x:v>
+        <x:v>full_primary_overlap.v5_primary_distinct_events_reached_from_v3_primary</x:v>
       </x:c>
       <x:c r="D77" s="71" t="n">
-        <x:v>2</x:v>
+        <x:v>774</x:v>
       </x:c>
       <x:c r="E77" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F77" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G77" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19014,22 +19014,22 @@
         <x:v>FRAME-77</x:v>
       </x:c>
       <x:c r="B78" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C78" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.now_zero_completed_substantive_action.v4_primary_ce</x:v>
+        <x:v>full_primary_overlap.v5_primary_events_not_reached_from_v3_primary</x:v>
       </x:c>
       <x:c r="D78" s="71" t="n">
-        <x:v>3</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="E78" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F78" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G78" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19037,22 +19037,22 @@
         <x:v>FRAME-78</x:v>
       </x:c>
       <x:c r="B79" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C79" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.now_zero_completed_substantive_action.v4_primary_comparison</x:v>
+        <x:v>full_primary_overlap.v5_primary_member_count</x:v>
       </x:c>
       <x:c r="D79" s="71" t="n">
-        <x:v>5</x:v>
+        <x:v>776</x:v>
       </x:c>
       <x:c r="E79" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F79" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G79" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19060,68 +19060,68 @@
         <x:v>FRAME-79</x:v>
       </x:c>
       <x:c r="B80" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C80" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.now_zero_completed_substantive_action.v4_resolved</x:v>
+        <x:v>full_primary_overlap.v5_primary_total</x:v>
       </x:c>
       <x:c r="D80" s="71" t="n">
-        <x:v>107</x:v>
+        <x:v>858</x:v>
       </x:c>
       <x:c r="E80" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F80" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G80" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="81" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A81" s="7" t="str">
         <x:v>FRAME-80</x:v>
       </x:c>
       <x:c r="B81" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C81" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.now_zero_completed_substantive_action.v4_unrestricted_ce</x:v>
+        <x:v>full_primary_overlap.disposition_counts.current_primary_changed</x:v>
       </x:c>
       <x:c r="D81" s="71" t="n">
-        <x:v>15</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="E81" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F81" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G81" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="82" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; unchanged/changed uses substantive tracked-evidence equality, excluding status-only transitions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A82" s="7" t="str">
         <x:v>FRAME-81</x:v>
       </x:c>
       <x:c r="B82" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C82" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.now_zero_completed_substantive_action.v4_unrestricted_comparison</x:v>
+        <x:v>full_primary_overlap.disposition_counts.current_primary_unchanged</x:v>
       </x:c>
       <x:c r="D82" s="71" t="n">
-        <x:v>21</x:v>
+        <x:v>629</x:v>
       </x:c>
       <x:c r="E82" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F82" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G82" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; unchanged/changed uses substantive tracked-evidence equality, excluding status-only transitions</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19129,22 +19129,22 @@
         <x:v>FRAME-82</x:v>
       </x:c>
       <x:c r="B83" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C83" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.reference_count_changed.v4_primary_ce</x:v>
+        <x:v>full_primary_overlap.disposition_counts.held</x:v>
       </x:c>
       <x:c r="D83" s="71" t="n">
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E83" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F83" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G83" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19152,45 +19152,45 @@
         <x:v>FRAME-83</x:v>
       </x:c>
       <x:c r="B84" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C84" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.reference_count_changed.v4_resolved</x:v>
+        <x:v>full_primary_overlap.disposition_counts.not_current_primary</x:v>
       </x:c>
       <x:c r="D84" s="71" t="n">
-        <x:v>128</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="E84" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F84" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G84" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="85" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A85" s="7" t="str">
         <x:v>FRAME-84</x:v>
       </x:c>
       <x:c r="B85" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C85" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.reference_count_changed.v4_unrestricted_ce</x:v>
+        <x:v>full_primary_overlap.change_category_counts.alias_membership_change_without_measurement_or_label_change</x:v>
       </x:c>
       <x:c r="D85" s="71" t="n">
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E85" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F85" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G85" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; mutually exclusive priority: derived labels, source measurements, aliases, status-only, strictly unchanged</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -19198,22 +19198,22 @@
         <x:v>FRAME-85</x:v>
       </x:c>
       <x:c r="B86" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C86" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.route_or_status_changed.v4_primary_ce</x:v>
+        <x:v>full_primary_overlap.change_category_counts.derived_label_change</x:v>
       </x:c>
       <x:c r="D86" s="71" t="n">
-        <x:v>4</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="E86" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F86" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G86" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components; changes in analysis.cohort() eligibility/condition or resolved/held status, not bare automated_disposition</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; mutually exclusive priority: derived labels, source measurements, aliases, status-only, strictly unchanged</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -19221,22 +19221,22 @@
         <x:v>FRAME-86</x:v>
       </x:c>
       <x:c r="B87" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C87" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.route_or_status_changed.v4_primary_comparison</x:v>
+        <x:v>full_primary_overlap.change_category_counts.measurement_change_without_derived_label_change</x:v>
       </x:c>
       <x:c r="D87" s="71" t="n">
-        <x:v>15</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E87" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F87" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G87" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components; changes in analysis.cohort() eligibility/condition or resolved/held status, not bare automated_disposition</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; mutually exclusive priority: derived labels, source measurements, aliases, status-only, strictly unchanged</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -19244,45 +19244,45 @@
         <x:v>FRAME-87</x:v>
       </x:c>
       <x:c r="B88" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C88" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.route_or_status_changed.v4_resolved</x:v>
+        <x:v>full_primary_overlap.change_category_counts.provenance_status_only</x:v>
       </x:c>
       <x:c r="D88" s="71" t="n">
-        <x:v>252</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="E88" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F88" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G88" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components; changes in analysis.cohort() eligibility/condition or resolved/held status, not bare automated_disposition</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="89" ht="52.79999923706055" hidden="0" customHeight="1">
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; only provenance-status text changes; observed transition v2_codex_unchanged to resolved, with unchanged identity, aliases and tracked evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A89" s="7" t="str">
         <x:v>FRAME-88</x:v>
       </x:c>
       <x:c r="B89" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C89" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.route_or_status_changed.v4_unrestricted_ce</x:v>
+        <x:v>full_primary_overlap.change_category_counts.strictly_unchanged</x:v>
       </x:c>
       <x:c r="D89" s="71" t="n">
-        <x:v>16</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="E89" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F89" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G89" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components; changes in analysis.cohort() eligibility/condition or resolved/held status, not bare automated_disposition</x:v>
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; strict equality includes exact provenance-status text, not just substantive evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -19290,183 +19290,183 @@
         <x:v>FRAME-89</x:v>
       </x:c>
       <x:c r="B90" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C90" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.route_or_status_changed.v4_unrestricted_comparison</x:v>
+        <x:v>full_primary_overlap.current_primary_change_category_counts.alias_membership_change_without_measurement_or_label_change</x:v>
       </x:c>
       <x:c r="D90" s="71" t="n">
-        <x:v>59</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E90" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F90" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G90" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components; changes in analysis.cohort() eligibility/condition or resolved/held status, not bare automated_disposition</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="91" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; mutually exclusive priority: derived labels, source measurements, aliases, status-only, strictly unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A91" s="7" t="str">
         <x:v>FRAME-90</x:v>
       </x:c>
       <x:c r="B91" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C91" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.successful_todowrite_calls.v4_primary_ce</x:v>
+        <x:v>full_primary_overlap.current_primary_change_category_counts.derived_label_change</x:v>
       </x:c>
       <x:c r="D91" s="71" t="n">
-        <x:v>132</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="E91" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F91" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G91" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="92" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; mutually exclusive priority: derived labels, source measurements, aliases, status-only, strictly unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A92" s="7" t="str">
         <x:v>FRAME-91</x:v>
       </x:c>
       <x:c r="B92" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C92" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.successful_todowrite_calls.v4_primary_comparison</x:v>
+        <x:v>full_primary_overlap.current_primary_change_category_counts.measurement_change_without_derived_label_change</x:v>
       </x:c>
       <x:c r="D92" s="71" t="n">
-        <x:v>161</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="E92" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F92" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G92" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="93" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; mutually exclusive priority: derived labels, source measurements, aliases, status-only, strictly unchanged</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A93" s="7" t="str">
         <x:v>FRAME-92</x:v>
       </x:c>
       <x:c r="B93" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C93" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.successful_todowrite_calls.v4_resolved</x:v>
+        <x:v>full_primary_overlap.current_primary_change_category_counts.provenance_status_only</x:v>
       </x:c>
       <x:c r="D93" s="71" t="n">
-        <x:v>6726</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="E93" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F93" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G93" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="94" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; only provenance-status text changes; observed transition v2_codex_unchanged to resolved, with unchanged identity, aliases and tracked evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A94" s="7" t="str">
         <x:v>FRAME-93</x:v>
       </x:c>
       <x:c r="B94" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical to current primary overlap</x:v>
       </x:c>
       <x:c r="C94" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.successful_todowrite_calls.v4_unrestricted_ce</x:v>
+        <x:v>full_primary_overlap.current_primary_change_category_counts.strictly_unchanged</x:v>
       </x:c>
       <x:c r="D94" s="71" t="n">
-        <x:v>525</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="E94" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F94" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G94" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="95" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Distinguish historical event memberships from distinct current events; balancing can change membership; strict equality includes exact provenance-status text, not just substantive evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="15" hidden="0" customHeight="1">
       <x:c r="A95" s="7" t="str">
         <x:v>FRAME-94</x:v>
       </x:c>
       <x:c r="B95" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical operational evidence rejoin</x:v>
       </x:c>
       <x:c r="C95" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.successful_todowrite_calls.v4_unrestricted_comparison</x:v>
+        <x:v>historical_evidence_all138.distinct_v5_events</x:v>
       </x:c>
       <x:c r="D95" s="71" t="n">
-        <x:v>534</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="E95" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F95" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G95" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="96" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Operational evidence, not a representative classifier reference study</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="15" hidden="0" customHeight="1">
       <x:c r="A96" s="7" t="str">
         <x:v>FRAME-95</x:v>
       </x:c>
       <x:c r="B96" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical operational evidence rejoin</x:v>
       </x:c>
       <x:c r="C96" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.successful_todowrite_events.v4_primary_ce</x:v>
+        <x:v>historical_evidence_all138.distinct_v5_primary_events</x:v>
       </x:c>
       <x:c r="D96" s="71" t="n">
-        <x:v>34</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E96" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F96" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G96" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="97" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Operational evidence, not a representative classifier reference study</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="15" hidden="0" customHeight="1">
       <x:c r="A97" s="7" t="str">
         <x:v>FRAME-96</x:v>
       </x:c>
       <x:c r="B97" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical operational evidence rejoin</x:v>
       </x:c>
       <x:c r="C97" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.successful_todowrite_events.v4_primary_comparison</x:v>
+        <x:v>historical_evidence_all138.historical_records</x:v>
       </x:c>
       <x:c r="D97" s="71" t="n">
-        <x:v>49</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="E97" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F97" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G97" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
+        <x:v>Operational evidence, not a representative classifier reference study</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19474,22 +19474,22 @@
         <x:v>FRAME-97</x:v>
       </x:c>
       <x:c r="B98" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>historical operational evidence rejoin</x:v>
       </x:c>
       <x:c r="C98" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.successful_todowrite_events.v4_resolved</x:v>
+        <x:v>historical_evidence_all138.historical_records_mapping_to_v5_primary</x:v>
       </x:c>
       <x:c r="D98" s="71" t="n">
-        <x:v>1503</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E98" s="7" t="str">
         <x:v>count</x:v>
       </x:c>
       <x:c r="F98" s="7" t="str">
-        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+        <x:v>analysis/results/boundary_correction_summary.json</x:v>
       </x:c>
       <x:c r="G98" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
+        <x:v>Operational evidence, not a representative classifier reference study</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19497,13 +19497,13 @@
         <x:v>FRAME-98</x:v>
       </x:c>
       <x:c r="B99" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>event-v4 to event-v5 native identity accounting</x:v>
       </x:c>
       <x:c r="C99" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.successful_todowrite_events.v4_unrestricted_ce</x:v>
+        <x:v>invariants.native_invariant_checks</x:v>
       </x:c>
       <x:c r="D99" s="71" t="n">
-        <x:v>145</x:v>
+        <x:v>3948491</x:v>
       </x:c>
       <x:c r="E99" s="7" t="str">
         <x:v>count</x:v>
@@ -19512,7 +19512,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G99" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19520,13 +19520,13 @@
         <x:v>FRAME-99</x:v>
       </x:c>
       <x:c r="B100" s="7" t="str">
-        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
+        <x:v>event-v4 to event-v5 native identity accounting</x:v>
       </x:c>
       <x:c r="C100" s="7" t="str">
-        <x:v>fixed_v4_selection_exposure.successful_todowrite_events.v4_unrestricted_comparison</x:v>
+        <x:v>invariants.unchanged_native_event_identities</x:v>
       </x:c>
       <x:c r="D100" s="71" t="n">
-        <x:v>153</x:v>
+        <x:v>20965</x:v>
       </x:c>
       <x:c r="E100" s="7" t="str">
         <x:v>count</x:v>
@@ -19535,7 +19535,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G100" s="7" t="str">
-        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19543,13 +19543,13 @@
         <x:v>FRAME-100</x:v>
       </x:c>
       <x:c r="B101" s="7" t="str">
-        <x:v>event-v4 to event-v5 balanced membership</x:v>
+        <x:v>event-v4 to event-v5 automated disposition</x:v>
       </x:c>
       <x:c r="C101" s="7" t="str">
-        <x:v>sample_membership.primary.newly_selected_events</x:v>
+        <x:v>status_transitions.quarantined-&gt;quarantined</x:v>
       </x:c>
       <x:c r="D101" s="71" t="n">
-        <x:v>69</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="E101" s="7" t="str">
         <x:v>count</x:v>
@@ -19566,13 +19566,13 @@
         <x:v>FRAME-101</x:v>
       </x:c>
       <x:c r="B102" s="7" t="str">
-        <x:v>event-v4 to event-v5 balanced membership</x:v>
+        <x:v>event-v4 to event-v5 automated disposition</x:v>
       </x:c>
       <x:c r="C102" s="7" t="str">
-        <x:v>sample_membership.primary.removed_events</x:v>
+        <x:v>status_transitions.resolved-&gt;resolved</x:v>
       </x:c>
       <x:c r="D102" s="71" t="n">
-        <x:v>21</x:v>
+        <x:v>20682</x:v>
       </x:c>
       <x:c r="E102" s="7" t="str">
         <x:v>count</x:v>
@@ -19589,13 +19589,13 @@
         <x:v>FRAME-102</x:v>
       </x:c>
       <x:c r="B103" s="7" t="str">
-        <x:v>event-v4 to event-v5 balanced membership</x:v>
+        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
       </x:c>
       <x:c r="C103" s="7" t="str">
-        <x:v>sample_membership.primary.retained_changed_condition</x:v>
+        <x:v>measurement_changes.automated_disposition_changed_events</x:v>
       </x:c>
       <x:c r="D103" s="71" t="n">
-        <x:v>0</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="E103" s="7" t="str">
         <x:v>count</x:v>
@@ -19604,7 +19604,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G103" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19612,13 +19612,13 @@
         <x:v>FRAME-103</x:v>
       </x:c>
       <x:c r="B104" s="7" t="str">
-        <x:v>event-v4 to event-v5 balanced membership</x:v>
+        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
       </x:c>
       <x:c r="C104" s="7" t="str">
-        <x:v>sample_membership.primary.retained_distinct_events</x:v>
+        <x:v>measurement_changes.completed_substantive_action_calls_changed_events</x:v>
       </x:c>
       <x:c r="D104" s="71" t="n">
-        <x:v>789</x:v>
+        <x:v>1522</x:v>
       </x:c>
       <x:c r="E104" s="7" t="str">
         <x:v>count</x:v>
@@ -19627,7 +19627,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G104" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19635,13 +19635,13 @@
         <x:v>FRAME-104</x:v>
       </x:c>
       <x:c r="B105" s="7" t="str">
-        <x:v>event-v4 to event-v5 balanced membership</x:v>
+        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
       </x:c>
       <x:c r="C105" s="7" t="str">
-        <x:v>sample_membership.primary.retained_same_condition</x:v>
+        <x:v>measurement_changes.context_mode_mask_changed_events</x:v>
       </x:c>
       <x:c r="D105" s="71" t="n">
-        <x:v>789</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="E105" s="7" t="str">
         <x:v>count</x:v>
@@ -19650,7 +19650,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G105" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19658,13 +19658,13 @@
         <x:v>FRAME-105</x:v>
       </x:c>
       <x:c r="B106" s="7" t="str">
-        <x:v>event-v4 to event-v5 balanced membership</x:v>
+        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
       </x:c>
       <x:c r="C106" s="7" t="str">
-        <x:v>sample_membership.primary.v4_total</x:v>
+        <x:v>measurement_changes.context_trace_status_changed_events</x:v>
       </x:c>
       <x:c r="D106" s="71" t="n">
-        <x:v>810</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="E106" s="7" t="str">
         <x:v>count</x:v>
@@ -19673,7 +19673,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G106" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19681,13 +19681,13 @@
         <x:v>FRAME-106</x:v>
       </x:c>
       <x:c r="B107" s="7" t="str">
-        <x:v>event-v4 to event-v5 balanced membership</x:v>
+        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
       </x:c>
       <x:c r="C107" s="7" t="str">
-        <x:v>sample_membership.primary.v5_total</x:v>
+        <x:v>measurement_changes.frontloading_changed_events</x:v>
       </x:c>
       <x:c r="D107" s="71" t="n">
-        <x:v>858</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E107" s="7" t="str">
         <x:v>count</x:v>
@@ -19696,7 +19696,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G107" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19704,13 +19704,13 @@
         <x:v>FRAME-107</x:v>
       </x:c>
       <x:c r="B108" s="7" t="str">
-        <x:v>event-v4 to event-v5 balanced membership</x:v>
+        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
       </x:c>
       <x:c r="C108" s="7" t="str">
-        <x:v>sample_membership.unrestricted.newly_selected_events</x:v>
+        <x:v>measurement_changes.prompt_artifact_reference_count_changed_events</x:v>
       </x:c>
       <x:c r="D108" s="71" t="n">
-        <x:v>294</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="E108" s="7" t="str">
         <x:v>count</x:v>
@@ -19719,7 +19719,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G108" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19727,13 +19727,13 @@
         <x:v>FRAME-108</x:v>
       </x:c>
       <x:c r="B109" s="7" t="str">
-        <x:v>event-v4 to event-v5 balanced membership</x:v>
+        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
       </x:c>
       <x:c r="C109" s="7" t="str">
-        <x:v>sample_membership.unrestricted.removed_events</x:v>
+        <x:v>measurement_changes.reclassified_calls</x:v>
       </x:c>
       <x:c r="D109" s="71" t="n">
-        <x:v>50</x:v>
+        <x:v>6788</x:v>
       </x:c>
       <x:c r="E109" s="7" t="str">
         <x:v>count</x:v>
@@ -19742,7 +19742,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G109" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19750,13 +19750,13 @@
         <x:v>FRAME-109</x:v>
       </x:c>
       <x:c r="B110" s="7" t="str">
-        <x:v>event-v4 to event-v5 balanced membership</x:v>
+        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
       </x:c>
       <x:c r="C110" s="7" t="str">
-        <x:v>sample_membership.unrestricted.retained_changed_condition</x:v>
+        <x:v>measurement_changes.successful_reclassified_calls</x:v>
       </x:c>
       <x:c r="D110" s="71" t="n">
-        <x:v>39</x:v>
+        <x:v>6780</x:v>
       </x:c>
       <x:c r="E110" s="7" t="str">
         <x:v>count</x:v>
@@ -19765,7 +19765,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G110" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19773,13 +19773,13 @@
         <x:v>FRAME-110</x:v>
       </x:c>
       <x:c r="B111" s="7" t="str">
-        <x:v>event-v4 to event-v5 balanced membership</x:v>
+        <x:v>event-v4 to event-v5 rule-derived changes</x:v>
       </x:c>
       <x:c r="C111" s="7" t="str">
-        <x:v>sample_membership.unrestricted.retained_distinct_events</x:v>
+        <x:v>measurement_changes.successful_todowrite_events</x:v>
       </x:c>
       <x:c r="D111" s="71" t="n">
-        <x:v>2160</x:v>
+        <x:v>1522</x:v>
       </x:c>
       <x:c r="E111" s="7" t="str">
         <x:v>count</x:v>
@@ -19788,7 +19788,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G111" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>All normalized native components, including resolved and held events; not only the resolved analysis input</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19796,13 +19796,13 @@
         <x:v>FRAME-111</x:v>
       </x:c>
       <x:c r="B112" s="7" t="str">
-        <x:v>event-v4 to event-v5 balanced membership</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C112" s="7" t="str">
-        <x:v>sample_membership.unrestricted.retained_same_condition</x:v>
+        <x:v>fixed_v4_selection_exposure.frontloading_changed.v4_primary_ce</x:v>
       </x:c>
       <x:c r="D112" s="71" t="n">
-        <x:v>2121</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E112" s="7" t="str">
         <x:v>count</x:v>
@@ -19811,7 +19811,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G112" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19819,13 +19819,13 @@
         <x:v>FRAME-112</x:v>
       </x:c>
       <x:c r="B113" s="7" t="str">
-        <x:v>event-v4 to event-v5 balanced membership</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C113" s="7" t="str">
-        <x:v>sample_membership.unrestricted.v4_total</x:v>
+        <x:v>fixed_v4_selection_exposure.frontloading_changed.v4_resolved</x:v>
       </x:c>
       <x:c r="D113" s="71" t="n">
-        <x:v>2210</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E113" s="7" t="str">
         <x:v>count</x:v>
@@ -19834,7 +19834,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G113" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19842,13 +19842,13 @@
         <x:v>FRAME-113</x:v>
       </x:c>
       <x:c r="B114" s="7" t="str">
-        <x:v>event-v4 to event-v5 balanced membership</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C114" s="7" t="str">
-        <x:v>sample_membership.unrestricted.v5_total</x:v>
+        <x:v>fixed_v4_selection_exposure.frontloading_changed.v4_unrestricted_ce</x:v>
       </x:c>
       <x:c r="D114" s="71" t="n">
-        <x:v>2454</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E114" s="7" t="str">
         <x:v>count</x:v>
@@ -19857,7 +19857,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G114" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19865,13 +19865,13 @@
         <x:v>FRAME-114</x:v>
       </x:c>
       <x:c r="B115" s="7" t="str">
-        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C115" s="7" t="str">
-        <x:v>source_accounting.v4.canonical_resolved_sources</x:v>
+        <x:v>fixed_v4_selection_exposure.now_zero_completed_substantive_action.v4_primary_ce</x:v>
       </x:c>
       <x:c r="D115" s="71" t="n">
-        <x:v>4677</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E115" s="7" t="str">
         <x:v>count</x:v>
@@ -19880,7 +19880,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G115" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19888,13 +19888,13 @@
         <x:v>FRAME-115</x:v>
       </x:c>
       <x:c r="B116" s="7" t="str">
-        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C116" s="7" t="str">
-        <x:v>source_accounting.v4.contributing_alias_sources</x:v>
+        <x:v>fixed_v4_selection_exposure.now_zero_completed_substantive_action.v4_primary_comparison</x:v>
       </x:c>
       <x:c r="D116" s="71" t="n">
-        <x:v>4760</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E116" s="7" t="str">
         <x:v>count</x:v>
@@ -19903,7 +19903,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G116" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19911,13 +19911,13 @@
         <x:v>FRAME-116</x:v>
       </x:c>
       <x:c r="B117" s="7" t="str">
-        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C117" s="7" t="str">
-        <x:v>source_accounting.v4.contributing_not_canonical_resolved</x:v>
+        <x:v>fixed_v4_selection_exposure.now_zero_completed_substantive_action.v4_resolved</x:v>
       </x:c>
       <x:c r="D117" s="71" t="n">
-        <x:v>83</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E117" s="7" t="str">
         <x:v>count</x:v>
@@ -19926,7 +19926,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G117" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19934,13 +19934,13 @@
         <x:v>FRAME-117</x:v>
       </x:c>
       <x:c r="B118" s="7" t="str">
-        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C118" s="7" t="str">
-        <x:v>source_accounting.v4.delta_canonical_held</x:v>
+        <x:v>fixed_v4_selection_exposure.now_zero_completed_substantive_action.v4_unrestricted_ce</x:v>
       </x:c>
       <x:c r="D118" s="71" t="n">
-        <x:v>1</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E118" s="7" t="str">
         <x:v>count</x:v>
@@ -19949,7 +19949,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G118" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19957,13 +19957,13 @@
         <x:v>FRAME-118</x:v>
       </x:c>
       <x:c r="B119" s="7" t="str">
-        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C119" s="7" t="str">
-        <x:v>source_accounting.v4.delta_only_held_alias</x:v>
+        <x:v>fixed_v4_selection_exposure.now_zero_completed_substantive_action.v4_unrestricted_comparison</x:v>
       </x:c>
       <x:c r="D119" s="71" t="n">
-        <x:v>0</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="E119" s="7" t="str">
         <x:v>count</x:v>
@@ -19972,7 +19972,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G119" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -19980,13 +19980,13 @@
         <x:v>FRAME-119</x:v>
       </x:c>
       <x:c r="B120" s="7" t="str">
-        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C120" s="7" t="str">
-        <x:v>source_accounting.v4.delta_with_held_alias</x:v>
+        <x:v>fixed_v4_selection_exposure.reference_count_changed.v4_primary_ce</x:v>
       </x:c>
       <x:c r="D120" s="71" t="n">
-        <x:v>13</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E120" s="7" t="str">
         <x:v>count</x:v>
@@ -19995,7 +19995,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G120" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -20003,13 +20003,13 @@
         <x:v>FRAME-120</x:v>
       </x:c>
       <x:c r="B121" s="7" t="str">
-        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C121" s="7" t="str">
-        <x:v>source_accounting.v4.delta_with_resolved_alias</x:v>
+        <x:v>fixed_v4_selection_exposure.reference_count_changed.v4_resolved</x:v>
       </x:c>
       <x:c r="D121" s="71" t="n">
-        <x:v>83</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E121" s="7" t="str">
         <x:v>count</x:v>
@@ -20018,7 +20018,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G121" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -20026,13 +20026,13 @@
         <x:v>FRAME-121</x:v>
       </x:c>
       <x:c r="B122" s="7" t="str">
-        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C122" s="7" t="str">
-        <x:v>source_accounting.v4.delta_without_any_canonical_role</x:v>
+        <x:v>fixed_v4_selection_exposure.reference_count_changed.v4_unrestricted_ce</x:v>
       </x:c>
       <x:c r="D122" s="71" t="n">
-        <x:v>82</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E122" s="7" t="str">
         <x:v>count</x:v>
@@ -20041,21 +20041,21 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G122" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="123" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A123" s="7" t="str">
         <x:v>FRAME-122</x:v>
       </x:c>
       <x:c r="B123" s="7" t="str">
-        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C123" s="7" t="str">
-        <x:v>source_accounting.v5.canonical_resolved_sources</x:v>
+        <x:v>fixed_v4_selection_exposure.route_or_status_changed.v4_primary_ce</x:v>
       </x:c>
       <x:c r="D123" s="71" t="n">
-        <x:v>4677</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E123" s="7" t="str">
         <x:v>count</x:v>
@@ -20064,21 +20064,21 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G123" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="124" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components; changes in analysis.cohort() eligibility/condition or resolved/held status, not bare automated_disposition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A124" s="7" t="str">
         <x:v>FRAME-123</x:v>
       </x:c>
       <x:c r="B124" s="7" t="str">
-        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C124" s="7" t="str">
-        <x:v>source_accounting.v5.contributing_alias_sources</x:v>
+        <x:v>fixed_v4_selection_exposure.route_or_status_changed.v4_primary_comparison</x:v>
       </x:c>
       <x:c r="D124" s="71" t="n">
-        <x:v>4760</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E124" s="7" t="str">
         <x:v>count</x:v>
@@ -20087,21 +20087,21 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G124" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="125" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components; changes in analysis.cohort() eligibility/condition or resolved/held status, not bare automated_disposition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A125" s="7" t="str">
         <x:v>FRAME-124</x:v>
       </x:c>
       <x:c r="B125" s="7" t="str">
-        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C125" s="7" t="str">
-        <x:v>source_accounting.v5.contributing_not_canonical_resolved</x:v>
+        <x:v>fixed_v4_selection_exposure.route_or_status_changed.v4_resolved</x:v>
       </x:c>
       <x:c r="D125" s="71" t="n">
-        <x:v>83</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="E125" s="7" t="str">
         <x:v>count</x:v>
@@ -20110,21 +20110,21 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G125" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="126" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components; changes in analysis.cohort() eligibility/condition or resolved/held status, not bare automated_disposition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A126" s="7" t="str">
         <x:v>FRAME-125</x:v>
       </x:c>
       <x:c r="B126" s="7" t="str">
-        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C126" s="7" t="str">
-        <x:v>source_accounting.v5.delta_canonical_held</x:v>
+        <x:v>fixed_v4_selection_exposure.route_or_status_changed.v4_unrestricted_ce</x:v>
       </x:c>
       <x:c r="D126" s="71" t="n">
-        <x:v>1</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E126" s="7" t="str">
         <x:v>count</x:v>
@@ -20133,21 +20133,21 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G126" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="127" ht="26.399999618530273" hidden="0" customHeight="1">
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components; changes in analysis.cohort() eligibility/condition or resolved/held status, not bare automated_disposition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A127" s="7" t="str">
         <x:v>FRAME-126</x:v>
       </x:c>
       <x:c r="B127" s="7" t="str">
-        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C127" s="7" t="str">
-        <x:v>source_accounting.v5.delta_only_held_alias</x:v>
+        <x:v>fixed_v4_selection_exposure.route_or_status_changed.v4_unrestricted_comparison</x:v>
       </x:c>
       <x:c r="D127" s="71" t="n">
-        <x:v>0</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="E127" s="7" t="str">
         <x:v>count</x:v>
@@ -20156,7 +20156,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G127" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components; changes in analysis.cohort() eligibility/condition or resolved/held status, not bare automated_disposition</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -20164,13 +20164,13 @@
         <x:v>FRAME-127</x:v>
       </x:c>
       <x:c r="B128" s="7" t="str">
-        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C128" s="7" t="str">
-        <x:v>source_accounting.v5.delta_with_held_alias</x:v>
+        <x:v>fixed_v4_selection_exposure.successful_todowrite_calls.v4_primary_ce</x:v>
       </x:c>
       <x:c r="D128" s="71" t="n">
-        <x:v>13</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="E128" s="7" t="str">
         <x:v>count</x:v>
@@ -20179,7 +20179,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G128" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -20187,13 +20187,13 @@
         <x:v>FRAME-128</x:v>
       </x:c>
       <x:c r="B129" s="7" t="str">
-        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C129" s="7" t="str">
-        <x:v>source_accounting.v5.delta_with_resolved_alias</x:v>
+        <x:v>fixed_v4_selection_exposure.successful_todowrite_calls.v4_primary_comparison</x:v>
       </x:c>
       <x:c r="D129" s="71" t="n">
-        <x:v>83</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="E129" s="7" t="str">
         <x:v>count</x:v>
@@ -20202,7 +20202,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G129" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -20210,13 +20210,13 @@
         <x:v>FRAME-129</x:v>
       </x:c>
       <x:c r="B130" s="7" t="str">
-        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C130" s="7" t="str">
-        <x:v>source_accounting.v5.delta_without_any_canonical_role</x:v>
+        <x:v>fixed_v4_selection_exposure.successful_todowrite_calls.v4_resolved</x:v>
       </x:c>
       <x:c r="D130" s="71" t="n">
-        <x:v>82</x:v>
+        <x:v>6726</x:v>
       </x:c>
       <x:c r="E130" s="7" t="str">
         <x:v>count</x:v>
@@ -20225,7 +20225,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G130" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -20233,13 +20233,13 @@
         <x:v>FRAME-130</x:v>
       </x:c>
       <x:c r="B131" s="7" t="str">
-        <x:v>resolved occurrences of unchanged administrative-tool candidates</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C131" s="7" t="str">
-        <x:v>unchanged_tool_names_resolved_occurrence_counts.v4.bashoutput</x:v>
+        <x:v>fixed_v4_selection_exposure.successful_todowrite_calls.v4_unrestricted_ce</x:v>
       </x:c>
       <x:c r="D131" s="71" t="n">
-        <x:v>0</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="E131" s="7" t="str">
         <x:v>count</x:v>
@@ -20248,7 +20248,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G131" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -20256,13 +20256,13 @@
         <x:v>FRAME-131</x:v>
       </x:c>
       <x:c r="B132" s="7" t="str">
-        <x:v>resolved occurrences of unchanged administrative-tool candidates</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C132" s="7" t="str">
-        <x:v>unchanged_tool_names_resolved_occurrence_counts.v4.killshell</x:v>
+        <x:v>fixed_v4_selection_exposure.successful_todowrite_calls.v4_unrestricted_comparison</x:v>
       </x:c>
       <x:c r="D132" s="71" t="n">
-        <x:v>0</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="E132" s="7" t="str">
         <x:v>count</x:v>
@@ -20271,7 +20271,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G132" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -20279,13 +20279,13 @@
         <x:v>FRAME-132</x:v>
       </x:c>
       <x:c r="B133" s="7" t="str">
-        <x:v>resolved occurrences of unchanged administrative-tool candidates</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C133" s="7" t="str">
-        <x:v>unchanged_tool_names_resolved_occurrence_counts.v5.bashoutput</x:v>
+        <x:v>fixed_v4_selection_exposure.successful_todowrite_events.v4_primary_ce</x:v>
       </x:c>
       <x:c r="D133" s="71" t="n">
-        <x:v>0</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="E133" s="7" t="str">
         <x:v>count</x:v>
@@ -20294,7 +20294,7 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G133" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
       </x:c>
     </x:row>
     <x:row r="134" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -20302,13 +20302,13 @@
         <x:v>FRAME-133</x:v>
       </x:c>
       <x:c r="B134" s="7" t="str">
-        <x:v>resolved occurrences of unchanged administrative-tool candidates</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C134" s="7" t="str">
-        <x:v>unchanged_tool_names_resolved_occurrence_counts.v5.killshell</x:v>
+        <x:v>fixed_v4_selection_exposure.successful_todowrite_events.v4_primary_comparison</x:v>
       </x:c>
       <x:c r="D134" s="71" t="n">
-        <x:v>0</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="E134" s="7" t="str">
         <x:v>count</x:v>
@@ -20317,21 +20317,21 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G134" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="135" ht="39.599998474121094" hidden="0" customHeight="1">
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A135" s="7" t="str">
         <x:v>FRAME-134</x:v>
       </x:c>
       <x:c r="B135" s="7" t="str">
-        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C135" s="7" t="str">
-        <x:v>phrase_overlap_exposure.counts.v4.eligible_ce_events</x:v>
+        <x:v>fixed_v4_selection_exposure.successful_todowrite_events.v4_resolved</x:v>
       </x:c>
       <x:c r="D135" s="71" t="n">
-        <x:v>0</x:v>
+        <x:v>1503</x:v>
       </x:c>
       <x:c r="E135" s="7" t="str">
         <x:v>count</x:v>
@@ -20340,21 +20340,21 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G135" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="136" ht="39.599998474121094" hidden="0" customHeight="1">
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A136" s="7" t="str">
         <x:v>FRAME-135</x:v>
       </x:c>
       <x:c r="B136" s="7" t="str">
-        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C136" s="7" t="str">
-        <x:v>phrase_overlap_exposure.counts.v4.eligible_comparison_events</x:v>
+        <x:v>fixed_v4_selection_exposure.successful_todowrite_events.v4_unrestricted_ce</x:v>
       </x:c>
       <x:c r="D136" s="71" t="n">
-        <x:v>0</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="E136" s="7" t="str">
         <x:v>count</x:v>
@@ -20363,21 +20363,21 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G136" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="137" ht="39.599998474121094" hidden="0" customHeight="1">
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A137" s="7" t="str">
         <x:v>FRAME-136</x:v>
       </x:c>
       <x:c r="B137" s="7" t="str">
-        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+        <x:v>changed measurements within fixed historical event-v4 selections</x:v>
       </x:c>
       <x:c r="C137" s="7" t="str">
-        <x:v>phrase_overlap_exposure.counts.v4.primary_events</x:v>
+        <x:v>fixed_v4_selection_exposure.successful_todowrite_events.v4_unrestricted_comparison</x:v>
       </x:c>
       <x:c r="D137" s="71" t="n">
-        <x:v>0</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="E137" s="7" t="str">
         <x:v>count</x:v>
@@ -20386,21 +20386,21 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G137" s="7" t="str">
-        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="138" ht="39.599998474121094" hidden="0" customHeight="1">
+        <x:v>Fixed historical v4 subset named in the measure; resolved subset excludes held components</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A138" s="7" t="str">
         <x:v>FRAME-137</x:v>
       </x:c>
       <x:c r="B138" s="7" t="str">
-        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+        <x:v>event-v4 to event-v5 balanced membership</x:v>
       </x:c>
       <x:c r="C138" s="7" t="str">
-        <x:v>phrase_overlap_exposure.counts.v4.resolved_events</x:v>
+        <x:v>sample_membership.primary.newly_selected_events</x:v>
       </x:c>
       <x:c r="D138" s="71" t="n">
-        <x:v>109</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="E138" s="7" t="str">
         <x:v>count</x:v>
@@ -20412,18 +20412,18 @@
         <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
       </x:c>
     </x:row>
-    <x:row r="139" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="139" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A139" s="7" t="str">
         <x:v>FRAME-138</x:v>
       </x:c>
       <x:c r="B139" s="7" t="str">
-        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+        <x:v>event-v4 to event-v5 balanced membership</x:v>
       </x:c>
       <x:c r="C139" s="7" t="str">
-        <x:v>phrase_overlap_exposure.counts.v4.sole_packaging_trigger_events</x:v>
+        <x:v>sample_membership.primary.removed_events</x:v>
       </x:c>
       <x:c r="D139" s="71" t="n">
-        <x:v>25</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="E139" s="7" t="str">
         <x:v>count</x:v>
@@ -20435,15 +20435,15 @@
         <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
       </x:c>
     </x:row>
-    <x:row r="140" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="140" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A140" s="7" t="str">
         <x:v>FRAME-139</x:v>
       </x:c>
       <x:c r="B140" s="7" t="str">
-        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+        <x:v>event-v4 to event-v5 balanced membership</x:v>
       </x:c>
       <x:c r="C140" s="7" t="str">
-        <x:v>phrase_overlap_exposure.counts.v4.unrestricted_events</x:v>
+        <x:v>sample_membership.primary.retained_changed_condition</x:v>
       </x:c>
       <x:c r="D140" s="71" t="n">
         <x:v>0</x:v>
@@ -20458,18 +20458,18 @@
         <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
       </x:c>
     </x:row>
-    <x:row r="141" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="141" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A141" s="7" t="str">
         <x:v>FRAME-140</x:v>
       </x:c>
       <x:c r="B141" s="7" t="str">
-        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+        <x:v>event-v4 to event-v5 balanced membership</x:v>
       </x:c>
       <x:c r="C141" s="7" t="str">
-        <x:v>phrase_overlap_exposure.counts.v5.eligible_ce_events</x:v>
+        <x:v>sample_membership.primary.retained_distinct_events</x:v>
       </x:c>
       <x:c r="D141" s="71" t="n">
-        <x:v>0</x:v>
+        <x:v>789</x:v>
       </x:c>
       <x:c r="E141" s="7" t="str">
         <x:v>count</x:v>
@@ -20481,18 +20481,18 @@
         <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
       </x:c>
     </x:row>
-    <x:row r="142" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="142" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A142" s="7" t="str">
         <x:v>FRAME-141</x:v>
       </x:c>
       <x:c r="B142" s="7" t="str">
-        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+        <x:v>event-v4 to event-v5 balanced membership</x:v>
       </x:c>
       <x:c r="C142" s="7" t="str">
-        <x:v>phrase_overlap_exposure.counts.v5.eligible_comparison_events</x:v>
+        <x:v>sample_membership.primary.retained_same_condition</x:v>
       </x:c>
       <x:c r="D142" s="71" t="n">
-        <x:v>0</x:v>
+        <x:v>789</x:v>
       </x:c>
       <x:c r="E142" s="7" t="str">
         <x:v>count</x:v>
@@ -20504,18 +20504,18 @@
         <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
       </x:c>
     </x:row>
-    <x:row r="143" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="143" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A143" s="7" t="str">
         <x:v>FRAME-142</x:v>
       </x:c>
       <x:c r="B143" s="7" t="str">
-        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+        <x:v>event-v4 to event-v5 balanced membership</x:v>
       </x:c>
       <x:c r="C143" s="7" t="str">
-        <x:v>phrase_overlap_exposure.counts.v5.primary_events</x:v>
+        <x:v>sample_membership.primary.v4_total</x:v>
       </x:c>
       <x:c r="D143" s="71" t="n">
-        <x:v>0</x:v>
+        <x:v>810</x:v>
       </x:c>
       <x:c r="E143" s="7" t="str">
         <x:v>count</x:v>
@@ -20527,18 +20527,18 @@
         <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
       </x:c>
     </x:row>
-    <x:row r="144" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="144" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A144" s="7" t="str">
         <x:v>FRAME-143</x:v>
       </x:c>
       <x:c r="B144" s="7" t="str">
-        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+        <x:v>event-v4 to event-v5 balanced membership</x:v>
       </x:c>
       <x:c r="C144" s="7" t="str">
-        <x:v>phrase_overlap_exposure.counts.v5.resolved_events</x:v>
+        <x:v>sample_membership.primary.v5_total</x:v>
       </x:c>
       <x:c r="D144" s="71" t="n">
-        <x:v>109</x:v>
+        <x:v>858</x:v>
       </x:c>
       <x:c r="E144" s="7" t="str">
         <x:v>count</x:v>
@@ -20550,18 +20550,18 @@
         <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
       </x:c>
     </x:row>
-    <x:row r="145" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="145" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A145" s="7" t="str">
         <x:v>FRAME-144</x:v>
       </x:c>
       <x:c r="B145" s="7" t="str">
-        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+        <x:v>event-v4 to event-v5 balanced membership</x:v>
       </x:c>
       <x:c r="C145" s="7" t="str">
-        <x:v>phrase_overlap_exposure.counts.v5.sole_packaging_trigger_events</x:v>
+        <x:v>sample_membership.unrestricted.newly_selected_events</x:v>
       </x:c>
       <x:c r="D145" s="71" t="n">
-        <x:v>25</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="E145" s="7" t="str">
         <x:v>count</x:v>
@@ -20573,18 +20573,18 @@
         <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
       </x:c>
     </x:row>
-    <x:row r="146" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="146" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A146" s="7" t="str">
         <x:v>FRAME-145</x:v>
       </x:c>
       <x:c r="B146" s="7" t="str">
-        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+        <x:v>event-v4 to event-v5 balanced membership</x:v>
       </x:c>
       <x:c r="C146" s="7" t="str">
-        <x:v>phrase_overlap_exposure.counts.v5.unrestricted_events</x:v>
+        <x:v>sample_membership.unrestricted.removed_events</x:v>
       </x:c>
       <x:c r="D146" s="71" t="n">
-        <x:v>0</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E146" s="7" t="str">
         <x:v>count</x:v>
@@ -20593,13 +20593,864 @@
         <x:v>analysis/results/action_reference_correction_summary.json</x:v>
       </x:c>
       <x:c r="G146" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A147" s="7" t="str">
+        <x:v>FRAME-146</x:v>
+      </x:c>
+      <x:c r="B147" s="7" t="str">
+        <x:v>event-v4 to event-v5 balanced membership</x:v>
+      </x:c>
+      <x:c r="C147" s="7" t="str">
+        <x:v>sample_membership.unrestricted.retained_changed_condition</x:v>
+      </x:c>
+      <x:c r="D147" s="7" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="E147" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F147" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G147" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A148" s="7" t="str">
+        <x:v>FRAME-147</x:v>
+      </x:c>
+      <x:c r="B148" s="7" t="str">
+        <x:v>event-v4 to event-v5 balanced membership</x:v>
+      </x:c>
+      <x:c r="C148" s="7" t="str">
+        <x:v>sample_membership.unrestricted.retained_distinct_events</x:v>
+      </x:c>
+      <x:c r="D148" s="7" t="n">
+        <x:v>2160</x:v>
+      </x:c>
+      <x:c r="E148" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F148" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G148" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A149" s="7" t="str">
+        <x:v>FRAME-148</x:v>
+      </x:c>
+      <x:c r="B149" s="7" t="str">
+        <x:v>event-v4 to event-v5 balanced membership</x:v>
+      </x:c>
+      <x:c r="C149" s="7" t="str">
+        <x:v>sample_membership.unrestricted.retained_same_condition</x:v>
+      </x:c>
+      <x:c r="D149" s="7" t="n">
+        <x:v>2121</x:v>
+      </x:c>
+      <x:c r="E149" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F149" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G149" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A150" s="7" t="str">
+        <x:v>FRAME-149</x:v>
+      </x:c>
+      <x:c r="B150" s="7" t="str">
+        <x:v>event-v4 to event-v5 balanced membership</x:v>
+      </x:c>
+      <x:c r="C150" s="7" t="str">
+        <x:v>sample_membership.unrestricted.v4_total</x:v>
+      </x:c>
+      <x:c r="D150" s="7" t="n">
+        <x:v>2210</x:v>
+      </x:c>
+      <x:c r="E150" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F150" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G150" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A151" s="7" t="str">
+        <x:v>FRAME-150</x:v>
+      </x:c>
+      <x:c r="B151" s="7" t="str">
+        <x:v>event-v4 to event-v5 balanced membership</x:v>
+      </x:c>
+      <x:c r="C151" s="7" t="str">
+        <x:v>sample_membership.unrestricted.v5_total</x:v>
+      </x:c>
+      <x:c r="D151" s="7" t="n">
+        <x:v>2454</x:v>
+      </x:c>
+      <x:c r="E151" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F151" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G151" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A152" s="7" t="str">
+        <x:v>FRAME-151</x:v>
+      </x:c>
+      <x:c r="B152" s="7" t="str">
+        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+      </x:c>
+      <x:c r="C152" s="7" t="str">
+        <x:v>source_accounting.v4.canonical_resolved_sources</x:v>
+      </x:c>
+      <x:c r="D152" s="7" t="n">
+        <x:v>4677</x:v>
+      </x:c>
+      <x:c r="E152" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F152" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G152" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A153" s="7" t="str">
+        <x:v>FRAME-152</x:v>
+      </x:c>
+      <x:c r="B153" s="7" t="str">
+        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+      </x:c>
+      <x:c r="C153" s="7" t="str">
+        <x:v>source_accounting.v4.contributing_alias_sources</x:v>
+      </x:c>
+      <x:c r="D153" s="7" t="n">
+        <x:v>4760</x:v>
+      </x:c>
+      <x:c r="E153" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F153" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G153" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A154" s="7" t="str">
+        <x:v>FRAME-153</x:v>
+      </x:c>
+      <x:c r="B154" s="7" t="str">
+        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+      </x:c>
+      <x:c r="C154" s="7" t="str">
+        <x:v>source_accounting.v4.contributing_not_canonical_resolved</x:v>
+      </x:c>
+      <x:c r="D154" s="7" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="E154" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F154" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G154" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A155" s="7" t="str">
+        <x:v>FRAME-154</x:v>
+      </x:c>
+      <x:c r="B155" s="7" t="str">
+        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+      </x:c>
+      <x:c r="C155" s="7" t="str">
+        <x:v>source_accounting.v4.delta_canonical_held</x:v>
+      </x:c>
+      <x:c r="D155" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E155" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F155" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G155" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A156" s="7" t="str">
+        <x:v>FRAME-155</x:v>
+      </x:c>
+      <x:c r="B156" s="7" t="str">
+        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+      </x:c>
+      <x:c r="C156" s="7" t="str">
+        <x:v>source_accounting.v4.delta_only_held_alias</x:v>
+      </x:c>
+      <x:c r="D156" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E156" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F156" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G156" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A157" s="7" t="str">
+        <x:v>FRAME-156</x:v>
+      </x:c>
+      <x:c r="B157" s="7" t="str">
+        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+      </x:c>
+      <x:c r="C157" s="7" t="str">
+        <x:v>source_accounting.v4.delta_with_held_alias</x:v>
+      </x:c>
+      <x:c r="D157" s="7" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E157" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F157" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G157" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A158" s="7" t="str">
+        <x:v>FRAME-157</x:v>
+      </x:c>
+      <x:c r="B158" s="7" t="str">
+        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+      </x:c>
+      <x:c r="C158" s="7" t="str">
+        <x:v>source_accounting.v4.delta_with_resolved_alias</x:v>
+      </x:c>
+      <x:c r="D158" s="7" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="E158" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F158" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G158" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A159" s="7" t="str">
+        <x:v>FRAME-158</x:v>
+      </x:c>
+      <x:c r="B159" s="7" t="str">
+        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+      </x:c>
+      <x:c r="C159" s="7" t="str">
+        <x:v>source_accounting.v4.delta_without_any_canonical_role</x:v>
+      </x:c>
+      <x:c r="D159" s="7" t="n">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="E159" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F159" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G159" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A160" s="7" t="str">
+        <x:v>FRAME-159</x:v>
+      </x:c>
+      <x:c r="B160" s="7" t="str">
+        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+      </x:c>
+      <x:c r="C160" s="7" t="str">
+        <x:v>source_accounting.v5.canonical_resolved_sources</x:v>
+      </x:c>
+      <x:c r="D160" s="7" t="n">
+        <x:v>4677</x:v>
+      </x:c>
+      <x:c r="E160" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F160" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G160" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A161" s="7" t="str">
+        <x:v>FRAME-160</x:v>
+      </x:c>
+      <x:c r="B161" s="7" t="str">
+        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+      </x:c>
+      <x:c r="C161" s="7" t="str">
+        <x:v>source_accounting.v5.contributing_alias_sources</x:v>
+      </x:c>
+      <x:c r="D161" s="7" t="n">
+        <x:v>4760</x:v>
+      </x:c>
+      <x:c r="E161" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F161" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G161" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A162" s="7" t="str">
+        <x:v>FRAME-161</x:v>
+      </x:c>
+      <x:c r="B162" s="7" t="str">
+        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+      </x:c>
+      <x:c r="C162" s="7" t="str">
+        <x:v>source_accounting.v5.contributing_not_canonical_resolved</x:v>
+      </x:c>
+      <x:c r="D162" s="7" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="E162" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F162" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G162" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A163" s="7" t="str">
+        <x:v>FRAME-162</x:v>
+      </x:c>
+      <x:c r="B163" s="7" t="str">
+        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+      </x:c>
+      <x:c r="C163" s="7" t="str">
+        <x:v>source_accounting.v5.delta_canonical_held</x:v>
+      </x:c>
+      <x:c r="D163" s="7" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E163" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F163" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G163" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A164" s="7" t="str">
+        <x:v>FRAME-163</x:v>
+      </x:c>
+      <x:c r="B164" s="7" t="str">
+        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+      </x:c>
+      <x:c r="C164" s="7" t="str">
+        <x:v>source_accounting.v5.delta_only_held_alias</x:v>
+      </x:c>
+      <x:c r="D164" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E164" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F164" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G164" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A165" s="7" t="str">
+        <x:v>FRAME-164</x:v>
+      </x:c>
+      <x:c r="B165" s="7" t="str">
+        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+      </x:c>
+      <x:c r="C165" s="7" t="str">
+        <x:v>source_accounting.v5.delta_with_held_alias</x:v>
+      </x:c>
+      <x:c r="D165" s="7" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E165" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F165" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G165" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A166" s="7" t="str">
+        <x:v>FRAME-165</x:v>
+      </x:c>
+      <x:c r="B166" s="7" t="str">
+        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+      </x:c>
+      <x:c r="C166" s="7" t="str">
+        <x:v>source_accounting.v5.delta_with_resolved_alias</x:v>
+      </x:c>
+      <x:c r="D166" s="7" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="E166" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F166" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G166" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A167" s="7" t="str">
+        <x:v>FRAME-166</x:v>
+      </x:c>
+      <x:c r="B167" s="7" t="str">
+        <x:v>contributing alias sources versus canonical resolved sources</x:v>
+      </x:c>
+      <x:c r="C167" s="7" t="str">
+        <x:v>source_accounting.v5.delta_without_any_canonical_role</x:v>
+      </x:c>
+      <x:c r="D167" s="7" t="n">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="E167" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F167" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G167" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A168" s="7" t="str">
+        <x:v>FRAME-167</x:v>
+      </x:c>
+      <x:c r="B168" s="7" t="str">
+        <x:v>resolved occurrences of unchanged administrative-tool candidates</x:v>
+      </x:c>
+      <x:c r="C168" s="7" t="str">
+        <x:v>unchanged_tool_names_resolved_occurrence_counts.v4.bashoutput</x:v>
+      </x:c>
+      <x:c r="D168" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E168" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F168" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G168" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A169" s="7" t="str">
+        <x:v>FRAME-168</x:v>
+      </x:c>
+      <x:c r="B169" s="7" t="str">
+        <x:v>resolved occurrences of unchanged administrative-tool candidates</x:v>
+      </x:c>
+      <x:c r="C169" s="7" t="str">
+        <x:v>unchanged_tool_names_resolved_occurrence_counts.v4.killshell</x:v>
+      </x:c>
+      <x:c r="D169" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E169" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F169" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G169" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A170" s="7" t="str">
+        <x:v>FRAME-169</x:v>
+      </x:c>
+      <x:c r="B170" s="7" t="str">
+        <x:v>resolved occurrences of unchanged administrative-tool candidates</x:v>
+      </x:c>
+      <x:c r="C170" s="7" t="str">
+        <x:v>unchanged_tool_names_resolved_occurrence_counts.v5.bashoutput</x:v>
+      </x:c>
+      <x:c r="D170" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E170" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F170" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G170" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A171" s="7" t="str">
+        <x:v>FRAME-170</x:v>
+      </x:c>
+      <x:c r="B171" s="7" t="str">
+        <x:v>resolved occurrences of unchanged administrative-tool candidates</x:v>
+      </x:c>
+      <x:c r="C171" s="7" t="str">
+        <x:v>unchanged_tool_names_resolved_occurrence_counts.v5.killshell</x:v>
+      </x:c>
+      <x:c r="D171" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E171" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F171" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G171" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A172" s="7" t="str">
+        <x:v>FRAME-171</x:v>
+      </x:c>
+      <x:c r="B172" s="7" t="str">
+        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+      </x:c>
+      <x:c r="C172" s="7" t="str">
+        <x:v>phrase_overlap_exposure.counts.v4.eligible_ce_events</x:v>
+      </x:c>
+      <x:c r="D172" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E172" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F172" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G172" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A173" s="7" t="str">
+        <x:v>FRAME-172</x:v>
+      </x:c>
+      <x:c r="B173" s="7" t="str">
+        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+      </x:c>
+      <x:c r="C173" s="7" t="str">
+        <x:v>phrase_overlap_exposure.counts.v4.eligible_comparison_events</x:v>
+      </x:c>
+      <x:c r="D173" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E173" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F173" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G173" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A174" s="7" t="str">
+        <x:v>FRAME-173</x:v>
+      </x:c>
+      <x:c r="B174" s="7" t="str">
+        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+      </x:c>
+      <x:c r="C174" s="7" t="str">
+        <x:v>phrase_overlap_exposure.counts.v4.primary_events</x:v>
+      </x:c>
+      <x:c r="D174" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E174" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F174" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G174" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A175" s="7" t="str">
+        <x:v>FRAME-174</x:v>
+      </x:c>
+      <x:c r="B175" s="7" t="str">
+        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+      </x:c>
+      <x:c r="C175" s="7" t="str">
+        <x:v>phrase_overlap_exposure.counts.v4.resolved_events</x:v>
+      </x:c>
+      <x:c r="D175" s="7" t="n">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="E175" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F175" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G175" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A176" s="7" t="str">
+        <x:v>FRAME-175</x:v>
+      </x:c>
+      <x:c r="B176" s="7" t="str">
+        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+      </x:c>
+      <x:c r="C176" s="7" t="str">
+        <x:v>phrase_overlap_exposure.counts.v4.sole_packaging_trigger_events</x:v>
+      </x:c>
+      <x:c r="D176" s="7" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="E176" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F176" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G176" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A177" s="7" t="str">
+        <x:v>FRAME-176</x:v>
+      </x:c>
+      <x:c r="B177" s="7" t="str">
+        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+      </x:c>
+      <x:c r="C177" s="7" t="str">
+        <x:v>phrase_overlap_exposure.counts.v4.unrestricted_events</x:v>
+      </x:c>
+      <x:c r="D177" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E177" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F177" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G177" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A178" s="7" t="str">
+        <x:v>FRAME-177</x:v>
+      </x:c>
+      <x:c r="B178" s="7" t="str">
+        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+      </x:c>
+      <x:c r="C178" s="7" t="str">
+        <x:v>phrase_overlap_exposure.counts.v5.eligible_ce_events</x:v>
+      </x:c>
+      <x:c r="D178" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E178" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F178" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G178" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A179" s="7" t="str">
+        <x:v>FRAME-178</x:v>
+      </x:c>
+      <x:c r="B179" s="7" t="str">
+        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+      </x:c>
+      <x:c r="C179" s="7" t="str">
+        <x:v>phrase_overlap_exposure.counts.v5.eligible_comparison_events</x:v>
+      </x:c>
+      <x:c r="D179" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E179" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F179" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G179" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A180" s="7" t="str">
+        <x:v>FRAME-179</x:v>
+      </x:c>
+      <x:c r="B180" s="7" t="str">
+        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+      </x:c>
+      <x:c r="C180" s="7" t="str">
+        <x:v>phrase_overlap_exposure.counts.v5.primary_events</x:v>
+      </x:c>
+      <x:c r="D180" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E180" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F180" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G180" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A181" s="7" t="str">
+        <x:v>FRAME-180</x:v>
+      </x:c>
+      <x:c r="B181" s="7" t="str">
+        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+      </x:c>
+      <x:c r="C181" s="7" t="str">
+        <x:v>phrase_overlap_exposure.counts.v5.resolved_events</x:v>
+      </x:c>
+      <x:c r="D181" s="7" t="n">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="E181" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F181" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G181" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A182" s="7" t="str">
+        <x:v>FRAME-181</x:v>
+      </x:c>
+      <x:c r="B182" s="7" t="str">
+        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+      </x:c>
+      <x:c r="C182" s="7" t="str">
+        <x:v>phrase_overlap_exposure.counts.v5.sole_packaging_trigger_events</x:v>
+      </x:c>
+      <x:c r="D182" s="7" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="E182" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F182" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G182" s="7" t="str">
+        <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A183" s="7" t="str">
+        <x:v>FRAME-182</x:v>
+      </x:c>
+      <x:c r="B183" s="7" t="str">
+        <x:v>literal context-package phrase exposure, not semantic stage adjudication</x:v>
+      </x:c>
+      <x:c r="C183" s="7" t="str">
+        <x:v>phrase_overlap_exposure.counts.v5.unrestricted_events</x:v>
+      </x:c>
+      <x:c r="D183" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E183" s="7" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="F183" s="7" t="str">
+        <x:v>analysis/results/action_reference_correction_summary.json</x:v>
+      </x:c>
+      <x:c r="G183" s="7" t="str">
         <x:v>Computational correction accounting; no new human judgments or independent accuracy estimate</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd2ff040df804d96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf82e2a141f494f82"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43652,7 +44503,7 @@
       <x:c r="M322" s="38"/>
       <x:c r="N322" s="37"/>
       <x:c r="O322" s="37" t="n">
-        <x:v>0.7265625</x:v>
+        <x:v>0.726171875</x:v>
       </x:c>
       <x:c r="P322" s="37"/>
       <x:c r="Q322" s="37"/>
@@ -43666,13 +44517,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="Y322" s="38" t="n">
-        <x:v>1860</x:v>
+        <x:v>1859</x:v>
       </x:c>
       <x:c r="Z322" s="38" t="n">
         <x:v>2560</x:v>
       </x:c>
       <x:c r="AA322" s="38" t="n">
-        <x:v>700</x:v>
+        <x:v>701</x:v>
       </x:c>
       <x:c r="AB322" s="13" t="str">
         <x:v>analysis/results/inheritance_window_sensitivity.csv</x:v>
@@ -43715,7 +44566,7 @@
       <x:c r="M323" s="38"/>
       <x:c r="N323" s="37"/>
       <x:c r="O323" s="37" t="n">
-        <x:v>0.821875</x:v>
+        <x:v>0.821484375</x:v>
       </x:c>
       <x:c r="P323" s="37"/>
       <x:c r="Q323" s="37"/>
@@ -43729,13 +44580,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="Y323" s="38" t="n">
-        <x:v>2104</x:v>
+        <x:v>2103</x:v>
       </x:c>
       <x:c r="Z323" s="38" t="n">
         <x:v>2560</x:v>
       </x:c>
       <x:c r="AA323" s="38" t="n">
-        <x:v>456</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="AB323" s="13" t="str">
         <x:v>analysis/results/inheritance_window_sensitivity.csv</x:v>
@@ -44022,7 +44873,7 @@
       <x:c r="M328" s="38"/>
       <x:c r="N328" s="37"/>
       <x:c r="O328" s="38" t="n">
-        <x:v>1107</x:v>
+        <x:v>1106</x:v>
       </x:c>
       <x:c r="P328" s="37"/>
       <x:c r="Q328" s="37"/>
@@ -44077,7 +44928,7 @@
       <x:c r="M329" s="38"/>
       <x:c r="N329" s="37"/>
       <x:c r="O329" s="38" t="n">
-        <x:v>1149</x:v>
+        <x:v>1150</x:v>
       </x:c>
       <x:c r="P329" s="37"/>
       <x:c r="Q329" s="37"/>
@@ -44242,7 +45093,7 @@
       <x:c r="M332" s="38"/>
       <x:c r="N332" s="37"/>
       <x:c r="O332" s="38" t="n">
-        <x:v>907</x:v>
+        <x:v>909</x:v>
       </x:c>
       <x:c r="P332" s="37"/>
       <x:c r="Q332" s="37"/>
@@ -44407,7 +45258,7 @@
       <x:c r="M335" s="38"/>
       <x:c r="N335" s="37"/>
       <x:c r="O335" s="38" t="n">
-        <x:v>138</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="P335" s="37"/>
       <x:c r="Q335" s="37"/>
@@ -44462,7 +45313,7 @@
       <x:c r="M336" s="38"/>
       <x:c r="N336" s="37"/>
       <x:c r="O336" s="38" t="n">
-        <x:v>185</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="P336" s="37"/>
       <x:c r="Q336" s="37"/>
@@ -44598,7 +45449,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb965e886ee24f0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9c3719418134485"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>